<commit_message>
chore: configure gyyh oracle environment
</commit_message>
<xml_diff>
--- a/knowledge/config/test_config.xlsx
+++ b/knowledge/config/test_config.xlsx
@@ -605,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="27.81640625" customWidth="1" min="1" max="1"/>
@@ -638,7 +638,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>10.20.150.149</t>
+          <t>10.20.36.35</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -655,7 +655,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>10621</t>
+          <t>10370</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>handsome</t>
+          <t>Ifm30485%</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>基金:dxfund,信托:dxtrust,理财:fina,商养:dxcp</t>
+          <t>基金:dxfund,信托:dxtrust,理财:fina,商养:dxcp,商业养老金:dxcp,汇市通:hstc,保险:insure,个人养老金:per</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -723,12 +723,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>/home/lcpt60/lcpt_jar/lcpt-web-manager-dxfund/logs/</t>
+          <t>/home/ifm30/log/ifmmanage/</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>基金代销日志目录</t>
+          <t>统一日志目录</t>
         </is>
       </c>
     </row>
@@ -740,12 +740,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>/home/lcpt60/lcpt_jar/lcpt-web-manager-dxtrust/logs/</t>
+          <t>/home/ifm30/log/ifmmanage/</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>信托代销日志目录</t>
+          <t>统一日志目录</t>
         </is>
       </c>
     </row>
@@ -757,12 +757,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>/home/lcpt60/lcpt_jar/lcpt-web-manager-fina/logs/</t>
+          <t>/home/ifm30/log/ifmmanage/</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>理财代销日志目录</t>
+          <t>统一日志目录</t>
         </is>
       </c>
     </row>
@@ -774,12 +774,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>lcpt-manager.log</t>
+          <t>managestdout.log.20260612</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>主日志文件名（各模块通用）</t>
+          <t>主日志文件名（按今天日期）</t>
         </is>
       </c>
     </row>
@@ -791,12 +791,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>manager-stdout.log</t>
+          <t>managestdout.log.20260612</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>ShardingSphere分片查询日志文件</t>
+          <t>标准输出/SQL日志文件名（按今天日期）</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>http://10.20.150.149:10622/console/#/login</t>
+          <t>http://10.20.36.35:10371/ifmmanage/</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -945,12 +945,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ui_bc,ui_trust1,ui_fund1,ui_fina1,ui_dxcp1,ui_hstc1,ui_insure1,ui_per1</t>
+          <t>GYYHAUTO</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>table_db_mapping.json 涉及的数据库列表，逗号分隔。--build-mapping 和 --auto 时读取</t>
+          <t>table_db_mapping.json 涉及的数据库列表，逗号分隔</t>
         </is>
       </c>
     </row>
@@ -962,12 +962,114 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>/home/lcpt60/lcpt_jar/lcpt-web-manager-dxcp/logs/</t>
+          <t>/home/ifm30/log/ifmmanage/</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t>商业养老金日志目录</t>
+          <t>统一日志目录</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>log_path_hstc</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>/home/ifm30/log/ifmmanage/</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>统一日志目录</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>log_path_insure</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>/home/ifm30/log/ifmmanage/</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>统一日志目录</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>log_path_pension</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>/home/ifm30/log/ifmmanage/</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>统一日志目录</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>env_key</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>gyyh-auto</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>pytest --env=xxx 的值</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>single_db_key</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>GYYHAUTO</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>单库环境数据库 key</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>db_type</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>oracle</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>数据库类型</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: adapt agent for gyyh oracle environment
</commit_message>
<xml_diff>
--- a/knowledge/config/test_config.xlsx
+++ b/knowledge/config/test_config.xlsx
@@ -605,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="27.81640625" customWidth="1" min="1" max="1"/>
@@ -820,144 +820,155 @@
     <row r="13" ht="27.5" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>update_cache</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>缓存更新模块标识，[信托,公共,基金,商业养老金,理财] 用逗号分隔 填no则不更新</t>
+          <t>cdp_url</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>http://localhost:9222</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Chrome DevTools Protocol 地址</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>cdp_url</t>
+          <t>chrome_path</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>http://localhost:9222</t>
+          <t>C:\Program Files\Google\Chrome\Application\chrome.exe</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Chrome DevTools Protocol 地址</t>
+          <t>Chrome 可执行文件路径</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>chrome_path</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>C:\Program Files\Google\Chrome\Application\chrome.exe</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Chrome 可执行文件路径</t>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>branch_user</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>fh001</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>勘测登录账号</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>branch_user</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>fh003</t>
+          <t>branch_password</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>222222</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>勘测登录账号</t>
+          <t>勘测登录密码</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>branch_password</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="n">
-        <v>11111111</v>
+          <t>login_url</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>http://10.20.36.35:10371/ifmmanage/</t>
+        </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>勘测登录密码</t>
+          <t>登录地址</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>login_url</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>http://10.20.36.35:10371/ifmmanage/</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>登录地址</t>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>node_path</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>node的地址</t>
+          <t>db_mapping_dbs</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>GYYHAUTO</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>table_db_mapping.json 涉及的数据库列表，逗号分隔</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>owner</t>
+          <t>log_path_dxcp</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>wanghh49745</t>
+          <t>/home/ifm30/log/ifmmanage/</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>统一日志目录</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>db_mapping_dbs</t>
+          <t>log_path_hstc</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>GYYHAUTO</t>
+          <t>/home/ifm30/log/ifmmanage/</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>table_db_mapping.json 涉及的数据库列表，逗号分隔</t>
+          <t>统一日志目录</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>log_path_dxcp</t>
+          <t>log_path_insure</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -965,7 +976,7 @@
           <t>/home/ifm30/log/ifmmanage/</t>
         </is>
       </c>
-      <c r="C22" s="17" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>统一日志目录</t>
         </is>
@@ -974,7 +985,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>log_path_hstc</t>
+          <t>log_path_pension</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -991,83 +1002,49 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>log_path_insure</t>
+          <t>env_key</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>/home/ifm30/log/ifmmanage/</t>
+          <t>gyyh-auto</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>统一日志目录</t>
+          <t>pytest --env=xxx 的值</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>log_path_pension</t>
+          <t>single_db_key</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>/home/ifm30/log/ifmmanage/</t>
+          <t>GYYHAUTO</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>统一日志目录</t>
+          <t>单库环境数据库 key</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>env_key</t>
+          <t>db_type</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>gyyh-auto</t>
+          <t>oracle</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
-        <is>
-          <t>pytest --env=xxx 的值</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>single_db_key</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>GYYHAUTO</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>单库环境数据库 key</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>db_type</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>oracle</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
         <is>
           <t>数据库类型</t>
         </is>
@@ -1088,7 +1065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1133,479 +1110,1759 @@
       </c>
     </row>
     <row r="2" ht="14.5" customHeight="1">
-      <c r="A2" s="16" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>客户资料查询</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>客户资料</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>客户资料查询</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>客户销售商信息查询</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>客户资料</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>客户销售商信息查询</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>理财账户信息查询</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>客户资料</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>理财账户信息查询</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>登记银行账户信息查询</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>客户资料</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>登记银行账户信息查询</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>客户风险等级查询</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>客户资料</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>客户风险等级查询</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>客户风险评价答案查询</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>客户资料</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>客户风险评价答案查询</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>历史理财账户资料查询</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>客户资料</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>历史理财账户资料查询</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>客户号变更信息查询</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>客户资料</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>客户号变更信息查询</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>产品信息查询</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>产品信息查询</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>产品信息查询</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>产品额度信息查询</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>产品信息查询</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>产品额度信息查询</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>产品转换关系查询</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>产品信息查询</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>产品转换关系查询</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>理财中心文件查询</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>理财中心文件查询</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>理财中心文件查询</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>客户份额查询</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>份额查询</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>客户份额查询</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>客户份额明细查询</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>份额查询</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>客户份额明细查询</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>客户理财产品份额明细查询</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>份额查询</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>客户理财产品份额明细查询</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>理财产品份额变动流水查询</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>份额查询</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>理财产品份额变动流水查询</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>历史份额变动流水查询</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>份额查询</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>历史份额变动流水查询</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>定期定额申购协议查询</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>协议类查询</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>定期定额申购协议查询</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>定期定额申购协议留痕查询</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>协议类查询</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>定期定额申购协议留痕查询</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>历史定期定额申购协议查询</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>协议类查询</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>历史定期定额申购协议查询</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>周期滚动协议查询</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>协议类查询</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>周期滚动协议查询</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>账户类请求流水查询</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>当前交易流水</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>账户类请求流水查询</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>交易类请求流水查询</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>当前交易流水</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>交易类请求流水查询</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>实时交易请求汇总查询</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>当前交易流水</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>实时交易请求汇总查询</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>批量转联机交易请求流水查询</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>当前交易流水</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>批量转联机交易请求流水查询</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>账户类确认流水查询</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>历史交易流水</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>账户类确认流水查询</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>交易类确认流水查询</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>历史交易流水</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>交易类确认流水查询</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>历史账户类请求流水查询</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>历史交易流水</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>历史账户类请求流水查询</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>历史交易类请求流水查询</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>历史交易流水</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>历史交易类请求流水查询</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>冻结解冻流水查询</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>特殊流水查询</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>冻结解冻流水查询</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>试算不平记录查询</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>特殊流水查询</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>试算不平记录查询</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>申购赎回额度临时调整留痕查询</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>留痕查询</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>申购赎回额度临时调整留痕查询</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>黑名单命中情况查询</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>留痕查询</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>黑名单命中情况查询</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>申购赎回资金清算查询</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>滚续产品查询</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>申购赎回资金清算查询</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>历史份额变动查询</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>日日金查询</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>历史份额变动查询</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>当前份额变动查询</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>日日金查询</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>当前份额变动查询</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>申购交易流水查询</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>日日金查询</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>申购交易流水查询</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>申购交易确认流水查询</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>日日金查询</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>申购交易确认流水查询</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>赎回交易流水查询</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>日日金查询</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>赎回交易流水查询</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>赎回交易确认流水查询</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>日日金查询</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>赎回交易确认流水查询</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>wanghh49745</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>信托代销产品行情信息查询</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>信托代销</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>查询管理</t>
-        </is>
-      </c>
-      <c r="E2" s="12" t="inlineStr">
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>信托代销产品行情信息查询</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="16" t="inlineStr">
+    <row r="43">
+      <c r="A43" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>信托代销产品信息查询</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>信托代销</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>查询管理</t>
-        </is>
-      </c>
-      <c r="E3" s="12" t="inlineStr">
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>信托代销产品信息查询</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="16" t="inlineStr">
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>信托代销账户信息查询</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>信托代销</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>查询管理</t>
-        </is>
-      </c>
-      <c r="E4" s="12" t="inlineStr">
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>信托代销账户信息查询</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+    <row r="45">
+      <c r="A45" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>信托代销历史账户信息查询</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>信托代销</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>查询管理</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>信托代销历史账户信息查询</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>信托代销账户类请求流水查询</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>信托代销</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>查询管理</t>
-        </is>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>信托代销账户类请求流水查询</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>信托代销交易类请求流水查询</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>信托代销</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>查询管理</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
         <is>
           <t>信托代销交易类请求流水查询</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>信托代销当前冻结解冻流水查询</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>信托代销</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>查询管理</t>
-        </is>
-      </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>信托代销当前冻结解冻流水查询</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>信托代销历史冻结解冻流水查询</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>信托代销</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>查询管理</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>信托代销历史冻结解冻流水查询</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>信托代销历史冲正交易流水查询</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>信托代销</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>查询管理</t>
-        </is>
-      </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>信托代销历史冲正交易流水查询</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>信托代销冲正交易流水查询</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>信托代销</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>查询管理</t>
-        </is>
-      </c>
-      <c r="E11" s="12" t="inlineStr">
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
         <is>
           <t>信托代销冲正交易流水查询</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+    <row r="52">
+      <c r="A52" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>
       </c>
-      <c r="B12" s="19" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>商养服务费报表</t>
         </is>
       </c>
-      <c r="C12" s="16" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>商业养老金</t>
         </is>
       </c>
-      <c r="D12" s="15" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>报表管理</t>
         </is>
       </c>
-      <c r="E12" s="19" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>商养服务费报表</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
         <is>
           <t>基金代销频繁交易报表</t>
         </is>
       </c>
-      <c r="C13" s="16" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>基金代销</t>
         </is>
       </c>
-      <c r="D13" s="15" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>报表管理</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>基金代销频繁交易报表</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
         <is>
           <t>基金代销划款报表</t>
         </is>
       </c>
-      <c r="C14" s="16" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>基金代销</t>
         </is>
       </c>
-      <c r="D14" s="15" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>报表管理</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>基金代销划款报表</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-      <c r="B15" s="19" t="inlineStr">
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
         <is>
           <t>基金代销交易类确认流水查询</t>
         </is>
       </c>
-      <c r="C15" s="16" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>基金代销</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>查询管理</t>
-        </is>
-      </c>
-      <c r="E15" s="20" t="inlineStr">
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>基金代销交易类确认流水查询</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F55" t="inlineStr">
         <is>
           <t>wangjie25895</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
         <is>
           <t>基金代销频繁开销户报表</t>
         </is>
       </c>
-      <c r="C16" s="16" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>基金代销</t>
         </is>
       </c>
-      <c r="D16" s="15" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>报表管理</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>基金代销频繁开销户报表</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F56" t="inlineStr">
         <is>
           <t>chenzy39580</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
         <is>
           <t>基金代销产品涨幅报表</t>
         </is>
       </c>
-      <c r="C17" s="16" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>基金代销</t>
         </is>
       </c>
-      <c r="D17" s="15" t="inlineStr">
+      <c r="D57" t="inlineStr">
         <is>
           <t>报表管理</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>基金代销产品涨幅报表</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F57" t="inlineStr">
         <is>
           <t>zhengkf41824</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="15" t="inlineStr">
-        <is>
-          <t>未完成</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>未完成</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
         <is>
           <t>基金代销交易请求汇总-按TA</t>
         </is>
       </c>
-      <c r="C18" s="16" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>基金代销</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>查询管理</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>查询管理</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
         <is>
           <t>基金代销交易请求汇总-按TA</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F58" t="inlineStr">
         <is>
           <t>wangmq46773</t>
         </is>

</xml_diff>